<commit_message>
Flexible tables in PDF and configurations to include/exclude parts in the report (#117)
* make reports flex, add step 7, update colors

* add possibility to include optimize in report

* add dict from excel and only optimize when name

* Error in isnan fixed

* modified the excells with configs and add NEMO

* Same fix DSM but also for JSON en CSV

* add hardcoded page_dict functionality

---------

Co-authored-by: mike.verdaasdonk <mike.verdaasdonk@admin.pwc.com>
</commit_message>
<xml_diff>
--- a/src/vlinder/data/Beerwiser/xlsx/Beerwiser.xlsx
+++ b/src/vlinder/data/Beerwiser/xlsx/Beerwiser.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tdijk004/Documents/Tooling/vlinder/trbs/src/vlinder/data/Beerwiser/xlsx/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mverdaasdo001/Documents/Aangepast_report/trbs/src/vlinder/data/Beerwiser/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A29D46D-61FF-5144-9E3D-34F7F8E5FF3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE6D3D3-124D-7E4A-9694-B6D36F4ECACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1360" yWindow="1200" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="300" windowWidth="34560" windowHeight="20700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configurations" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="144">
   <si>
     <t>configuration</t>
   </si>
@@ -438,6 +438,45 @@
   </si>
   <si>
     <t>WURWE_sp</t>
+  </si>
+  <si>
+    <t>True</t>
+  </si>
+  <si>
+    <t>report_title_page</t>
+  </si>
+  <si>
+    <t>report_strategic_challenge</t>
+  </si>
+  <si>
+    <t>report_key_outputs_theme</t>
+  </si>
+  <si>
+    <t>report_decision_makers_options</t>
+  </si>
+  <si>
+    <t>report_scenarios</t>
+  </si>
+  <si>
+    <t>report_fixed_inputs</t>
+  </si>
+  <si>
+    <t>report_dependencies</t>
+  </si>
+  <si>
+    <t>report_weighted_appreciations</t>
+  </si>
+  <si>
+    <t>report_add_optimize</t>
+  </si>
+  <si>
+    <t>Optimize_DMO_name</t>
+  </si>
+  <si>
+    <t>False</t>
+  </si>
+  <si>
+    <t>Optimized_DMO</t>
   </si>
 </sst>
 </file>
@@ -551,8 +590,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1FD10895-72A3-7148-9AC0-E24F8F49DC8D}"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -852,10 +891,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -872,6 +912,86 @@
       </c>
       <c r="B2" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B12" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>